<commit_message>
updated file for entry
</commit_message>
<xml_diff>
--- a/files/Institutional_format.xlsx
+++ b/files/Institutional_format.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Q2026\Formats\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Aryabhat\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{602A92B7-57EA-48A7-A569-11E85865AF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9B65BA3-4FC8-442F-8AFB-838943CE8000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BFB9F8DC-31D7-49FC-91D7-3FC382DACE2E}"/>
   </bookViews>
@@ -295,9 +295,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="178" formatCode="dd\-mm\-yy"/>
-    <numFmt numFmtId="179" formatCode="dd\-mmm\-yy"/>
-    <numFmt numFmtId="181" formatCode="[$-409]dd/mmm/yy;@"/>
+    <numFmt numFmtId="164" formatCode="dd\-mm\-yy"/>
+    <numFmt numFmtId="165" formatCode="dd\-mmm\-yy"/>
+    <numFmt numFmtId="166" formatCode="[$-409]dd/mmm/yy;@"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -502,7 +502,7 @@
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
@@ -514,214 +514,165 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyProtection="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="181" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="15" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="179" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -737,7 +688,7 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -749,12 +700,61 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="15" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1088,34 +1088,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="20.25" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
       <c r="I1" s="1"/>
-      <c r="Z1" s="66" t="s">
+      <c r="Z1" s="34" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
       <c r="I2" s="1"/>
-      <c r="Z2" s="67" t="s">
+      <c r="Z2" s="35" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1129,39 +1129,39 @@
       <c r="G3" s="14"/>
       <c r="H3" s="16"/>
       <c r="I3" s="1"/>
-      <c r="Z3" s="67" t="s">
+      <c r="Z3" s="35" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="44" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="45"/>
+      <c r="G4" s="45"/>
+      <c r="H4" s="45"/>
       <c r="I4" s="1"/>
-      <c r="Z4" s="67" t="s">
+      <c r="Z4" s="35" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24"/>
+      <c r="B5" s="46"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="46"/>
       <c r="I5" s="1"/>
-      <c r="Z5" s="67" t="s">
+      <c r="Z5" s="35" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1175,237 +1175,239 @@
       <c r="G6" s="14"/>
       <c r="H6" s="16"/>
       <c r="I6" s="1"/>
-      <c r="Z6" s="67" t="s">
+      <c r="Z6" s="35" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="59"/>
-      <c r="C7" s="60"/>
-      <c r="D7" s="60"/>
-      <c r="E7" s="60"/>
-      <c r="F7" s="60"/>
-      <c r="G7" s="60"/>
-      <c r="H7" s="60"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="48"/>
+      <c r="H7" s="48"/>
       <c r="I7" s="1"/>
-      <c r="Z7" s="67" t="s">
+      <c r="Z7" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="61"/>
-      <c r="C8" s="60"/>
-      <c r="D8" s="60"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="62"/>
-      <c r="G8" s="58" t="s">
+      <c r="B8" s="49"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="48"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="50"/>
+      <c r="G8" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="H8" s="26"/>
+      <c r="H8" s="19"/>
       <c r="I8" s="1"/>
-      <c r="Z8" s="67" t="s">
+      <c r="Z8" s="35" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="63"/>
-      <c r="C9" s="64"/>
-      <c r="D9" s="64"/>
-      <c r="E9" s="65"/>
-      <c r="F9" s="27" t="s">
+      <c r="B9" s="51"/>
+      <c r="C9" s="52"/>
+      <c r="D9" s="52"/>
+      <c r="E9" s="53"/>
+      <c r="F9" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
+      <c r="G9" s="67"/>
+      <c r="H9" s="67"/>
       <c r="I9" s="1"/>
-      <c r="Z9" s="67" t="s">
+      <c r="Z9" s="35" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="63"/>
-      <c r="C10" s="64"/>
-      <c r="D10" s="64"/>
-      <c r="E10" s="64"/>
-      <c r="F10" s="64"/>
-      <c r="G10" s="64"/>
-      <c r="H10" s="64"/>
+      <c r="B10" s="51"/>
+      <c r="C10" s="52"/>
+      <c r="D10" s="52"/>
+      <c r="E10" s="52"/>
+      <c r="F10" s="52"/>
+      <c r="G10" s="52"/>
+      <c r="H10" s="52"/>
       <c r="I10" s="1"/>
-      <c r="Z10" s="67" t="s">
+      <c r="Z10" s="35" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A11" s="29"/>
-      <c r="B11" s="30"/>
-      <c r="C11" s="30"/>
-      <c r="D11" s="30"/>
-      <c r="E11" s="30"/>
-      <c r="F11" s="30"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="30"/>
+      <c r="A11" s="60"/>
+      <c r="B11" s="61"/>
+      <c r="C11" s="61"/>
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="61"/>
       <c r="I11" s="1"/>
-      <c r="Z11" s="67" t="s">
+      <c r="Z11" s="35" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A12" s="31" t="s">
+      <c r="A12" s="36" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="32"/>
-      <c r="C12" s="32"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="34"/>
-      <c r="G12" s="34"/>
-      <c r="H12" s="34"/>
+      <c r="B12" s="37"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="37"/>
+      <c r="E12" s="38"/>
+      <c r="F12" s="39"/>
+      <c r="G12" s="39"/>
+      <c r="H12" s="39"/>
       <c r="I12" s="1"/>
-      <c r="Z12" s="67" t="s">
+      <c r="Z12" s="35" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A13" s="31" t="s">
+      <c r="A13" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="32"/>
-      <c r="C13" s="32"/>
-      <c r="D13" s="32"/>
-      <c r="E13" s="33"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="34"/>
+      <c r="B13" s="37"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="37"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
+      <c r="H13" s="39"/>
       <c r="I13" s="1"/>
-      <c r="Z13" s="67" t="s">
+      <c r="Z13" s="35" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A14" s="35"/>
-      <c r="B14" s="36"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="38"/>
-      <c r="G14" s="37"/>
-      <c r="H14" s="38"/>
+      <c r="A14" s="21"/>
+      <c r="B14" s="23"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="24"/>
       <c r="I14" s="1"/>
-      <c r="Z14" s="67" t="s">
+      <c r="Z14" s="35" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A15" s="29" t="s">
+      <c r="A15" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="30"/>
-      <c r="C15" s="30"/>
-      <c r="D15" s="30"/>
-      <c r="E15" s="30"/>
-      <c r="F15" s="30"/>
-      <c r="G15" s="30"/>
-      <c r="H15" s="30"/>
+      <c r="B15" s="61"/>
+      <c r="C15" s="61"/>
+      <c r="D15" s="61"/>
+      <c r="E15" s="61"/>
+      <c r="F15" s="61"/>
+      <c r="G15" s="61"/>
+      <c r="H15" s="61"/>
       <c r="I15" s="1"/>
-      <c r="Z15" s="67" t="s">
+      <c r="Z15" s="35" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A16" s="39" t="s">
+      <c r="A16" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="40"/>
-      <c r="C16" s="41"/>
-      <c r="D16" s="39" t="s">
+      <c r="B16" s="62">
+        <v>46256</v>
+      </c>
+      <c r="C16" s="63"/>
+      <c r="D16" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="E16" s="42"/>
-      <c r="F16" s="43" t="s">
+      <c r="E16" s="27"/>
+      <c r="F16" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="G16" s="43"/>
-      <c r="H16" s="44"/>
+      <c r="G16" s="64"/>
+      <c r="H16" s="26"/>
       <c r="I16" s="1"/>
-      <c r="Z16" s="67" t="s">
+      <c r="Z16" s="35" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A17" s="45"/>
-      <c r="B17" s="46"/>
-      <c r="C17" s="46"/>
-      <c r="D17" s="46"/>
-      <c r="E17" s="46"/>
-      <c r="F17" s="46"/>
-      <c r="G17" s="46"/>
-      <c r="H17" s="46"/>
+      <c r="A17" s="65"/>
+      <c r="B17" s="66"/>
+      <c r="C17" s="66"/>
+      <c r="D17" s="66"/>
+      <c r="E17" s="66"/>
+      <c r="F17" s="66"/>
+      <c r="G17" s="66"/>
+      <c r="H17" s="66"/>
       <c r="I17" s="1"/>
-      <c r="Z17" s="67" t="s">
+      <c r="Z17" s="35" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A18" s="47" t="s">
+      <c r="A18" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="B18" s="48"/>
-      <c r="C18" s="49" t="s">
+      <c r="B18" s="55"/>
+      <c r="C18" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="50" t="s">
+      <c r="D18" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="E18" s="51" t="s">
+      <c r="E18" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="F18" s="52" t="s">
+      <c r="F18" s="56" t="s">
         <v>2</v>
       </c>
-      <c r="G18" s="53" t="s">
+      <c r="G18" s="58" t="s">
         <v>3</v>
       </c>
-      <c r="H18" s="52" t="s">
+      <c r="H18" s="56" t="s">
         <v>17</v>
       </c>
       <c r="I18" s="1"/>
-      <c r="Z18" s="67" t="s">
+      <c r="Z18" s="35" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:26" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A19" s="54" t="s">
+      <c r="A19" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="B19" s="54" t="s">
+      <c r="B19" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="54" t="s">
+      <c r="C19" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="D19" s="54" t="s">
+      <c r="D19" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="E19" s="55" t="s">
+      <c r="E19" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="F19" s="56"/>
-      <c r="G19" s="57"/>
-      <c r="H19" s="56"/>
+      <c r="F19" s="57"/>
+      <c r="G19" s="59"/>
+      <c r="H19" s="57"/>
       <c r="I19" s="1"/>
-      <c r="Z19" s="67" t="s">
+      <c r="Z19" s="35" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1419,7 +1421,7 @@
       <c r="G20" s="11"/>
       <c r="H20" s="12"/>
       <c r="I20" s="1"/>
-      <c r="Z20" s="67" t="s">
+      <c r="Z20" s="35" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1432,7 +1434,7 @@
       <c r="F21" s="10"/>
       <c r="G21" s="11"/>
       <c r="H21" s="12"/>
-      <c r="Z21" s="67" t="s">
+      <c r="Z21" s="35" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1445,7 +1447,7 @@
       <c r="F22" s="10"/>
       <c r="G22" s="11"/>
       <c r="H22" s="12"/>
-      <c r="Z22" s="67" t="s">
+      <c r="Z22" s="35" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1458,7 +1460,7 @@
       <c r="F23" s="10"/>
       <c r="G23" s="11"/>
       <c r="H23" s="12"/>
-      <c r="Z23" s="67" t="s">
+      <c r="Z23" s="35" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1471,7 +1473,7 @@
       <c r="F24" s="10"/>
       <c r="G24" s="11"/>
       <c r="H24" s="12"/>
-      <c r="Z24" s="67" t="s">
+      <c r="Z24" s="35" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1484,7 +1486,7 @@
       <c r="F25" s="10"/>
       <c r="G25" s="11"/>
       <c r="H25" s="12"/>
-      <c r="Z25" s="67" t="s">
+      <c r="Z25" s="35" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1497,7 +1499,7 @@
       <c r="F26" s="10"/>
       <c r="G26" s="11"/>
       <c r="H26" s="12"/>
-      <c r="Z26" s="67" t="s">
+      <c r="Z26" s="35" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1510,7 +1512,7 @@
       <c r="F27" s="10"/>
       <c r="G27" s="11"/>
       <c r="H27" s="12"/>
-      <c r="Z27" s="67" t="s">
+      <c r="Z27" s="35" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1523,7 +1525,7 @@
       <c r="F28" s="10"/>
       <c r="G28" s="11"/>
       <c r="H28" s="12"/>
-      <c r="Z28" s="67" t="s">
+      <c r="Z28" s="35" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1536,7 +1538,7 @@
       <c r="F29" s="10"/>
       <c r="G29" s="11"/>
       <c r="H29" s="12"/>
-      <c r="Z29" s="67" t="s">
+      <c r="Z29" s="35" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1549,7 +1551,7 @@
       <c r="F30" s="10"/>
       <c r="G30" s="11"/>
       <c r="H30" s="12"/>
-      <c r="Z30" s="67" t="s">
+      <c r="Z30" s="35" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1562,7 +1564,7 @@
       <c r="F31" s="10"/>
       <c r="G31" s="11"/>
       <c r="H31" s="12"/>
-      <c r="Z31" s="67" t="s">
+      <c r="Z31" s="35" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1575,7 +1577,7 @@
       <c r="F32" s="10"/>
       <c r="G32" s="11"/>
       <c r="H32" s="12"/>
-      <c r="Z32" s="67" t="s">
+      <c r="Z32" s="35" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1588,7 +1590,7 @@
       <c r="F33" s="10"/>
       <c r="G33" s="11"/>
       <c r="H33" s="12"/>
-      <c r="Z33" s="67" t="s">
+      <c r="Z33" s="35" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1601,7 +1603,7 @@
       <c r="F34" s="10"/>
       <c r="G34" s="11"/>
       <c r="H34" s="12"/>
-      <c r="Z34" s="67" t="s">
+      <c r="Z34" s="35" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1614,7 +1616,7 @@
       <c r="F35" s="10"/>
       <c r="G35" s="11"/>
       <c r="H35" s="12"/>
-      <c r="Z35" s="67" t="s">
+      <c r="Z35" s="35" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1627,7 +1629,7 @@
       <c r="F36" s="10"/>
       <c r="G36" s="11"/>
       <c r="H36" s="12"/>
-      <c r="Z36" s="67" t="s">
+      <c r="Z36" s="35" t="s">
         <v>63</v>
       </c>
     </row>
@@ -1640,7 +1642,7 @@
       <c r="F37" s="10"/>
       <c r="G37" s="11"/>
       <c r="H37" s="12"/>
-      <c r="Z37" s="67" t="s">
+      <c r="Z37" s="35" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1653,7 +1655,7 @@
       <c r="F38" s="10"/>
       <c r="G38" s="11"/>
       <c r="H38" s="12"/>
-      <c r="Z38" s="67" t="s">
+      <c r="Z38" s="35" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1666,7 +1668,7 @@
       <c r="F39" s="10"/>
       <c r="G39" s="11"/>
       <c r="H39" s="12"/>
-      <c r="Z39" s="67" t="s">
+      <c r="Z39" s="35" t="s">
         <v>66</v>
       </c>
     </row>
@@ -1679,7 +1681,7 @@
       <c r="F40" s="10"/>
       <c r="G40" s="11"/>
       <c r="H40" s="12"/>
-      <c r="Z40" s="67" t="s">
+      <c r="Z40" s="35" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1692,7 +1694,7 @@
       <c r="F41" s="10"/>
       <c r="G41" s="11"/>
       <c r="H41" s="12"/>
-      <c r="Z41" s="67" t="s">
+      <c r="Z41" s="35" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1705,7 +1707,7 @@
       <c r="F42" s="10"/>
       <c r="G42" s="11"/>
       <c r="H42" s="12"/>
-      <c r="Z42" s="67" t="s">
+      <c r="Z42" s="35" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1718,7 +1720,7 @@
       <c r="F43" s="10"/>
       <c r="G43" s="11"/>
       <c r="H43" s="12"/>
-      <c r="Z43" s="67" t="s">
+      <c r="Z43" s="35" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1731,7 +1733,7 @@
       <c r="F44" s="10"/>
       <c r="G44" s="11"/>
       <c r="H44" s="12"/>
-      <c r="Z44" s="67" t="s">
+      <c r="Z44" s="35" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1744,7 +1746,7 @@
       <c r="F45" s="10"/>
       <c r="G45" s="11"/>
       <c r="H45" s="12"/>
-      <c r="Z45" s="67" t="s">
+      <c r="Z45" s="35" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1757,7 +1759,7 @@
       <c r="F46" s="10"/>
       <c r="G46" s="11"/>
       <c r="H46" s="12"/>
-      <c r="Z46" s="67" t="s">
+      <c r="Z46" s="35" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1770,7 +1772,7 @@
       <c r="F47" s="10"/>
       <c r="G47" s="11"/>
       <c r="H47" s="12"/>
-      <c r="Z47" s="67" t="s">
+      <c r="Z47" s="35" t="s">
         <v>74</v>
       </c>
     </row>
@@ -1783,7 +1785,7 @@
       <c r="F48" s="10"/>
       <c r="G48" s="11"/>
       <c r="H48" s="12"/>
-      <c r="Z48" s="67" t="s">
+      <c r="Z48" s="35" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1796,7 +1798,7 @@
       <c r="F49" s="10"/>
       <c r="G49" s="11"/>
       <c r="H49" s="12"/>
-      <c r="Z49" s="67" t="s">
+      <c r="Z49" s="35" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1809,7 +1811,7 @@
       <c r="F50" s="10"/>
       <c r="G50" s="11"/>
       <c r="H50" s="12"/>
-      <c r="Z50" s="67" t="s">
+      <c r="Z50" s="35" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1822,7 +1824,7 @@
       <c r="F51" s="10"/>
       <c r="G51" s="11"/>
       <c r="H51" s="12"/>
-      <c r="Z51" s="67" t="s">
+      <c r="Z51" s="35" t="s">
         <v>78</v>
       </c>
     </row>
@@ -1835,7 +1837,7 @@
       <c r="F52" s="10"/>
       <c r="G52" s="11"/>
       <c r="H52" s="12"/>
-      <c r="Z52" s="67" t="s">
+      <c r="Z52" s="35" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1848,7 +1850,7 @@
       <c r="F53" s="10"/>
       <c r="G53" s="11"/>
       <c r="H53" s="12"/>
-      <c r="Z53" s="67" t="s">
+      <c r="Z53" s="35" t="s">
         <v>80</v>
       </c>
     </row>
@@ -1861,7 +1863,7 @@
       <c r="F54" s="10"/>
       <c r="G54" s="11"/>
       <c r="H54" s="12"/>
-      <c r="Z54" s="67" t="s">
+      <c r="Z54" s="35" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1874,7 +1876,7 @@
       <c r="F55" s="10"/>
       <c r="G55" s="11"/>
       <c r="H55" s="12"/>
-      <c r="Z55" s="67" t="s">
+      <c r="Z55" s="35" t="s">
         <v>82</v>
       </c>
     </row>
@@ -1887,7 +1889,7 @@
       <c r="F56" s="10"/>
       <c r="G56" s="11"/>
       <c r="H56" s="12"/>
-      <c r="Z56" s="67" t="s">
+      <c r="Z56" s="35" t="s">
         <v>83</v>
       </c>
     </row>
@@ -21522,11 +21524,13 @@
       <c r="H2019" s="10"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="zZd17yZ8Y5H4/vM/r1Z7jJO/uMwogWdKn8AaB/DPfSia/HyUkm9M4nj+M9h4WQSuOoY2srslRUTICgYsdPal+A==" saltValue="q3878Y6w+wXF0c8LJWUnbA==" spinCount="100000" sheet="1" sort="0" autoFilter="0"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="vh5QRbEWj+J/sgcTP9tjg/Q66hFIh3I+eO464pXxGoZFkgxDxEnJaYi3WuqWf9o7QIpHYfTetgcs7pEjt/BqzA==" saltValue="CHjR8sZPXgjXnVsmayWn2Q==" spinCount="100000" sheet="1" sort="0" autoFilter="0"/>
   <mergeCells count="22">
-    <mergeCell ref="B7:H7"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="F13:H13"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="G9:H9"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="F18:F19"/>
     <mergeCell ref="G18:G19"/>
@@ -21535,32 +21539,30 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="A17:H17"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="F13:H13"/>
-    <mergeCell ref="A11:H11"/>
-    <mergeCell ref="B10:H10"/>
-    <mergeCell ref="G9:H9"/>
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="F12:H12"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B9:E9"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <dataValidations count="19">
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Network ???" error="Please enter only Yes or No" promptTitle="Network ???" prompt="Please indicate whether your computers are connected with each other through LAN" sqref="F13:H13" xr:uid="{AB8E9593-46B9-4C9C-B0D1-9DAD0302B60E}">
       <formula1>"Yes, No"</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Date 3" error="Quiz can be conducted between 1-Aug-18  and 3-Sep-18 only" promptTitle="Date 3" prompt="Enter your third choice of the date on which you desire to conduct the quiz at your school" sqref="H16" xr:uid="{C6C9BAEA-6810-4973-B7FC-C033DD8DC136}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Date 3" error="Quiz can be conducted between 1-Aug  and 3-Sep-2026 only" promptTitle="Date 3" prompt="Enter your third choice of the date as dd-mm-yyyy" sqref="H16" xr:uid="{C6C9BAEA-6810-4973-B7FC-C033DD8DC136}">
       <formula1>46235</formula1>
       <formula2>46268</formula2>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Date 2" error="Quiz can be conducted between 1-Aug-18  and 3-Sep-18 only" promptTitle="Date 2" prompt="Enter your second choice of the date on which you desire to conduct the quiz at your school" sqref="E16" xr:uid="{4103751A-5924-402D-96AD-053DCE86058D}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Date 2" error="Quiz can be conducted between 1-Aug  and 3-Sep-2026 only" promptTitle="Date 2" prompt="Enter your second choice of the date as dd-mm-yyyy" sqref="E16" xr:uid="{4103751A-5924-402D-96AD-053DCE86058D}">
       <formula1>46235</formula1>
       <formula2>46268</formula2>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Date" error="Quiz can be conducted between 1-Aug-18  and 3-Sep-18 only" promptTitle="Date 1" prompt="Enter your first choice of the date on which you desire to conduct the quiz at your school" sqref="B16:C16" xr:uid="{596339C4-5280-4049-B790-0DAFF17820FA}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Date" error="Quiz can be conducted between 1-Aug  and 3-Sep-2026 only" promptTitle="Date 1" prompt="Enter your first choice of the date as dd-mm-yyyy" sqref="B16:C16" xr:uid="{596339C4-5280-4049-B790-0DAFF17820FA}">
       <formula1>46235</formula1>
       <formula2>46268</formula2>
     </dataValidation>

</xml_diff>